<commit_message>
Add frontend fetal stage Kiwi
</commit_message>
<xml_diff>
--- a/frontend/data/source/AmazonNow_Dummy_Product_Dataset.xlsx
+++ b/frontend/data/source/AmazonNow_Dummy_Product_Dataset.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>Delivery_Time_Min</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Image_URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -473,6 +478,11 @@
       <c r="F2" t="n">
         <v>10</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1546470427-e26264be0b0d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -499,6 +509,11 @@
       <c r="F3" t="n">
         <v>10</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1518977676601-b53f82aba655?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -525,6 +540,11 @@
       <c r="F4" t="n">
         <v>10</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1587049633312-d628ae50a8ae?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -551,6 +571,11 @@
       <c r="F5" t="n">
         <v>10</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1571771894821-ce9b6c11b08e?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -577,6 +602,11 @@
       <c r="F6" t="n">
         <v>12</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1560806887-1e4cd0b6cbd6?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -603,6 +633,11 @@
       <c r="F7" t="n">
         <v>12</v>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1582979512210-99b6a53386f9?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -629,6 +664,11 @@
       <c r="F8" t="n">
         <v>10</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1445282768818-728615cc910a?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -655,6 +695,11 @@
       <c r="F9" t="n">
         <v>10</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1576045057995-568f588f82fb?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -681,6 +726,11 @@
       <c r="F10" t="n">
         <v>15</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1574323347407-f5e1ad6d020b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -707,6 +757,11 @@
       <c r="F11" t="n">
         <v>15</v>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1574323347407-f5e1ad6d020b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -733,6 +788,11 @@
       <c r="F12" t="n">
         <v>15</v>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1574323347407-f5e1ad6d020b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -759,6 +819,11 @@
       <c r="F13" t="n">
         <v>15</v>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1574323347407-f5e1ad6d020b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -785,6 +850,11 @@
       <c r="F14" t="n">
         <v>15</v>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1574323347407-f5e1ad6d020b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -811,6 +881,11 @@
       <c r="F15" t="n">
         <v>15</v>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1574323347407-f5e1ad6d020b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -837,6 +912,11 @@
       <c r="F16" t="n">
         <v>15</v>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1574323347407-f5e1ad6d020b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -863,6 +943,11 @@
       <c r="F17" t="n">
         <v>15</v>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1574323347407-f5e1ad6d020b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -889,6 +974,11 @@
       <c r="F18" t="n">
         <v>12</v>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1596040033229-a9821ebd058d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -915,6 +1005,11 @@
       <c r="F19" t="n">
         <v>12</v>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1596040033229-a9821ebd058d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -941,6 +1036,11 @@
       <c r="F20" t="n">
         <v>12</v>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1596040033229-a9821ebd058d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -967,6 +1067,11 @@
       <c r="F21" t="n">
         <v>12</v>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1596040033229-a9821ebd058d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -993,6 +1098,11 @@
       <c r="F22" t="n">
         <v>12</v>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1596040033229-a9821ebd058d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1019,6 +1129,11 @@
       <c r="F23" t="n">
         <v>12</v>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1596040033229-a9821ebd058d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1045,6 +1160,11 @@
       <c r="F24" t="n">
         <v>12</v>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1596040033229-a9821ebd058d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1071,6 +1191,11 @@
       <c r="F25" t="n">
         <v>12</v>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1596040033229-a9821ebd058d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1097,6 +1222,11 @@
       <c r="F26" t="n">
         <v>10</v>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1628088062854-d1870b4553da?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1123,6 +1253,11 @@
       <c r="F27" t="n">
         <v>10</v>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1628088062854-d1870b4553da?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1149,6 +1284,11 @@
       <c r="F28" t="n">
         <v>10</v>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1628088062854-d1870b4553da?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1175,6 +1315,11 @@
       <c r="F29" t="n">
         <v>10</v>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1628088062854-d1870b4553da?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1201,6 +1346,11 @@
       <c r="F30" t="n">
         <v>10</v>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1628088062854-d1870b4553da?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1227,6 +1377,11 @@
       <c r="F31" t="n">
         <v>10</v>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1589985270826-4b7bb135bc9d?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1253,6 +1408,11 @@
       <c r="F32" t="n">
         <v>10</v>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1628088062854-d1870b4553da?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1279,6 +1439,11 @@
       <c r="F33" t="n">
         <v>10</v>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1628088062854-d1870b4553da?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1305,6 +1470,11 @@
       <c r="F34" t="n">
         <v>10</v>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1509440159596-0249088772ff?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1331,6 +1501,11 @@
       <c r="F35" t="n">
         <v>10</v>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1509440159596-0249088772ff?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1357,6 +1532,11 @@
       <c r="F36" t="n">
         <v>10</v>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1509440159596-0249088772ff?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1383,6 +1563,11 @@
       <c r="F37" t="n">
         <v>10</v>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1509440159596-0249088772ff?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1409,6 +1594,11 @@
       <c r="F38" t="n">
         <v>10</v>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1509440159596-0249088772ff?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1435,6 +1625,11 @@
       <c r="F39" t="n">
         <v>10</v>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1509440159596-0249088772ff?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1461,6 +1656,11 @@
       <c r="F40" t="n">
         <v>10</v>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1509440159596-0249088772ff?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1487,6 +1687,11 @@
       <c r="F41" t="n">
         <v>10</v>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1509440159596-0249088772ff?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1513,6 +1718,11 @@
       <c r="F42" t="n">
         <v>12</v>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1517093157656-b9eccef91cb1?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1539,6 +1749,11 @@
       <c r="F43" t="n">
         <v>12</v>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1517093157656-b9eccef91cb1?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1565,6 +1780,11 @@
       <c r="F44" t="n">
         <v>12</v>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1517093157656-b9eccef91cb1?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1591,6 +1811,11 @@
       <c r="F45" t="n">
         <v>12</v>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1517093157656-b9eccef91cb1?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1617,6 +1842,11 @@
       <c r="F46" t="n">
         <v>12</v>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1517093157656-b9eccef91cb1?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1643,6 +1873,11 @@
       <c r="F47" t="n">
         <v>12</v>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1517093157656-b9eccef91cb1?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1669,6 +1904,11 @@
       <c r="F48" t="n">
         <v>12</v>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1517093157656-b9eccef91cb1?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1695,6 +1935,11 @@
       <c r="F49" t="n">
         <v>12</v>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1517093157656-b9eccef91cb1?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1721,6 +1966,11 @@
       <c r="F50" t="n">
         <v>15</v>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1607623814075-e51df1bdc82f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1747,6 +1997,11 @@
       <c r="F51" t="n">
         <v>15</v>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1607623814075-e51df1bdc82f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1773,6 +2028,11 @@
       <c r="F52" t="n">
         <v>15</v>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1607623814075-e51df1bdc82f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1799,6 +2059,11 @@
       <c r="F53" t="n">
         <v>15</v>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1607623814075-e51df1bdc82f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1825,6 +2090,11 @@
       <c r="F54" t="n">
         <v>15</v>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1607623814075-e51df1bdc82f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1851,6 +2121,11 @@
       <c r="F55" t="n">
         <v>15</v>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1607623814075-e51df1bdc82f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1877,6 +2152,11 @@
       <c r="F56" t="n">
         <v>15</v>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1607623814075-e51df1bdc82f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1903,6 +2183,11 @@
       <c r="F57" t="n">
         <v>15</v>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1607623814075-e51df1bdc82f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1929,6 +2214,11 @@
       <c r="F58" t="n">
         <v>20</v>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1556911220-bff31c812dba?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1955,6 +2245,11 @@
       <c r="F59" t="n">
         <v>20</v>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1556911220-bff31c812dba?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1981,6 +2276,11 @@
       <c r="F60" t="n">
         <v>20</v>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1556911220-bff31c812dba?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2007,6 +2307,11 @@
       <c r="F61" t="n">
         <v>20</v>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1556911220-bff31c812dba?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2033,6 +2338,11 @@
       <c r="F62" t="n">
         <v>20</v>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1556911220-bff31c812dba?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2059,6 +2369,11 @@
       <c r="F63" t="n">
         <v>20</v>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1556911220-bff31c812dba?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2085,6 +2400,11 @@
       <c r="F64" t="n">
         <v>10</v>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1566478989037-eec170784d0b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2111,6 +2431,11 @@
       <c r="F65" t="n">
         <v>10</v>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1566478989037-eec170784d0b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2137,6 +2462,11 @@
       <c r="F66" t="n">
         <v>10</v>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1566478989037-eec170784d0b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2163,6 +2493,11 @@
       <c r="F67" t="n">
         <v>10</v>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1566478989037-eec170784d0b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2189,6 +2524,11 @@
       <c r="F68" t="n">
         <v>10</v>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1549007994-cb92caebd54b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2215,6 +2555,11 @@
       <c r="F69" t="n">
         <v>10</v>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1549007994-cb92caebd54b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2241,6 +2586,11 @@
       <c r="F70" t="n">
         <v>10</v>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1549007994-cb92caebd54b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2267,6 +2617,11 @@
       <c r="F71" t="n">
         <v>10</v>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1549007994-cb92caebd54b?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2293,6 +2648,11 @@
       <c r="F72" t="n">
         <v>10</v>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1622483767028-3f66f32aef97?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2319,6 +2679,11 @@
       <c r="F73" t="n">
         <v>10</v>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1629203851122-3726ecdf080e?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2345,6 +2710,11 @@
       <c r="F74" t="n">
         <v>10</v>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1622597467836-f3285f2131b8?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2371,6 +2741,11 @@
       <c r="F75" t="n">
         <v>10</v>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1622597467836-f3285f2131b8?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2397,6 +2772,11 @@
       <c r="F76" t="n">
         <v>10</v>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1544787219-7f47ccb76574?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2423,6 +2803,11 @@
       <c r="F77" t="n">
         <v>10</v>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1514432324607-a09d9b4aefdd?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2449,6 +2834,11 @@
       <c r="F78" t="n">
         <v>10</v>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1544787219-7f47ccb76574?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2475,6 +2865,11 @@
       <c r="F79" t="n">
         <v>10</v>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1544787219-7f47ccb76574?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2501,6 +2896,11 @@
       <c r="F80" t="n">
         <v>10</v>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1626804475297-41608ea09aeb?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2527,6 +2927,11 @@
       <c r="F81" t="n">
         <v>10</v>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1626804475297-41608ea09aeb?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2553,6 +2958,11 @@
       <c r="F82" t="n">
         <v>12</v>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1579722821273-0f6c7d44362f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2579,6 +2989,11 @@
       <c r="F83" t="n">
         <v>12</v>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1579722821273-0f6c7d44362f?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2605,6 +3020,11 @@
       <c r="F84" t="n">
         <v>10</v>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1501443762994-82bd5dace89a?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2630,6 +3050,11 @@
       </c>
       <c r="F85" t="n">
         <v>10</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1563805042-7684c019e1cb?auto=format&amp;fit=crop&amp;w=500&amp;q=80</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>